<commit_message>
Increase chart margins and title size
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017beCMsx4BNYhXiiUzmNymi
</commit_message>
<xml_diff>
--- a/capabilities/economic-research/model.xlsx
+++ b/capabilities/economic-research/model.xlsx
@@ -144,16 +144,31 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1800" b="1"/>
             </a:pPr>
             <a:r>
+              <a:rPr sz="1800" b="1"/>
               <a:t>Number of deals</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <layoutTarget val="inner"/>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.13"/>
+          <y val="0.17"/>
+          <w val="0.82"/>
+          <h val="0.64"/>
+        </manualLayout>
+      </layout>
       <scatterChart>
         <ser>
           <idx val="0"/>
@@ -210,14 +225,16 @@
               <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
               <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
-                  <a:defRPr/>
+                  <a:defRPr sz="1100" b="1"/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr sz="1100" b="1"/>
                   <a:t>Year</a:t>
                 </a:r>
               </a:p>
             </rich>
           </tx>
+          <overlay val="0"/>
         </title>
         <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
@@ -238,17 +255,19 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" vert="horz"/>
               <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
-                  <a:defRPr/>
+                  <a:defRPr sz="1100" b="1"/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr sz="1100" b="1"/>
                   <a:t>Number of deals</a:t>
                 </a:r>
               </a:p>
             </rich>
           </tx>
+          <overlay val="0"/>
         </title>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
@@ -273,16 +292,31 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1800" b="1"/>
             </a:pPr>
             <a:r>
+              <a:rPr sz="1800" b="1"/>
               <a:t>Dollar amount financed (in million $)</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <layoutTarget val="inner"/>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.13"/>
+          <y val="0.17"/>
+          <w val="0.82"/>
+          <h val="0.64"/>
+        </manualLayout>
+      </layout>
       <scatterChart>
         <ser>
           <idx val="0"/>
@@ -339,14 +373,16 @@
               <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
               <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
-                  <a:defRPr/>
+                  <a:defRPr sz="1100" b="1"/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr sz="1100" b="1"/>
                   <a:t>Year</a:t>
                 </a:r>
               </a:p>
             </rich>
           </tx>
+          <overlay val="0"/>
         </title>
         <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
@@ -367,17 +403,19 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" vert="horz"/>
               <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
-                  <a:defRPr/>
+                  <a:defRPr sz="1100" b="1"/>
                 </a:pPr>
                 <a:r>
+                  <a:rPr sz="1100" b="1"/>
                   <a:t>USD millions</a:t>
                 </a:r>
               </a:p>
             </rich>
           </tx>
+          <overlay val="0"/>
         </title>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>

</xml_diff>